<commit_message>
Færdiggjort uge 37 og lavet odds til uge 38
</commit_message>
<xml_diff>
--- a/English Premier League/Raw/25_26.xlsx
+++ b/English Premier League/Raw/25_26.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP31"/>
+  <dimension ref="A1:AP41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3259,7 +3259,7 @@
         <v>7</v>
       </c>
       <c r="J21" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K21" t="n">
         <v>391</v>
@@ -3330,7 +3330,7 @@
         <v>13</v>
       </c>
       <c r="AG21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AH21" t="n">
         <v>17</v>
@@ -3351,13 +3351,13 @@
         <v>63</v>
       </c>
       <c r="AN21" t="n">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="AO21" t="n">
         <v>390</v>
       </c>
       <c r="AP21" t="n">
-        <v>81.59999999999999</v>
+        <v>81.8</v>
       </c>
     </row>
     <row r="22">
@@ -4718,6 +4718,1366 @@
       </c>
       <c r="AP31" t="n">
         <v>82.59999999999999</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" t="n">
+        <v>16</v>
+      </c>
+      <c r="F32" t="n">
+        <v>5</v>
+      </c>
+      <c r="G32" t="n">
+        <v>54</v>
+      </c>
+      <c r="H32" t="n">
+        <v>8</v>
+      </c>
+      <c r="I32" t="n">
+        <v>8</v>
+      </c>
+      <c r="J32" t="n">
+        <v>20</v>
+      </c>
+      <c r="K32" t="n">
+        <v>615</v>
+      </c>
+      <c r="L32" t="n">
+        <v>13</v>
+      </c>
+      <c r="M32" t="n">
+        <v>7</v>
+      </c>
+      <c r="N32" t="n">
+        <v>9</v>
+      </c>
+      <c r="O32" t="n">
+        <v>16</v>
+      </c>
+      <c r="P32" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>6</v>
+      </c>
+      <c r="R32" t="n">
+        <v>12</v>
+      </c>
+      <c r="S32" t="n">
+        <v>43</v>
+      </c>
+      <c r="T32" t="n">
+        <v>517</v>
+      </c>
+      <c r="U32" t="n">
+        <v>434</v>
+      </c>
+      <c r="V32" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>Nottingham Forest</t>
+        </is>
+      </c>
+      <c r="X32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>46</v>
+      </c>
+      <c r="AB32" t="n">
+        <v>11</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>13</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>544</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>12</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>11</v>
+      </c>
+      <c r="AH32" t="n">
+        <v>8</v>
+      </c>
+      <c r="AI32" t="n">
+        <v>20</v>
+      </c>
+      <c r="AJ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK32" t="n">
+        <v>11</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>23</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>56</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>448</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>373</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>83.3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Crystal Palace</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>14</v>
+      </c>
+      <c r="F33" t="n">
+        <v>6</v>
+      </c>
+      <c r="G33" t="n">
+        <v>56</v>
+      </c>
+      <c r="H33" t="n">
+        <v>10</v>
+      </c>
+      <c r="I33" t="n">
+        <v>5</v>
+      </c>
+      <c r="J33" t="n">
+        <v>20</v>
+      </c>
+      <c r="K33" t="n">
+        <v>639</v>
+      </c>
+      <c r="L33" t="n">
+        <v>10</v>
+      </c>
+      <c r="M33" t="n">
+        <v>6</v>
+      </c>
+      <c r="N33" t="n">
+        <v>14</v>
+      </c>
+      <c r="O33" t="n">
+        <v>27</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>8</v>
+      </c>
+      <c r="R33" t="n">
+        <v>23</v>
+      </c>
+      <c r="S33" t="n">
+        <v>76</v>
+      </c>
+      <c r="T33" t="n">
+        <v>539</v>
+      </c>
+      <c r="U33" t="n">
+        <v>439</v>
+      </c>
+      <c r="V33" t="n">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>Sunderland</t>
+        </is>
+      </c>
+      <c r="X33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>44</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>8</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>17</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>539</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>13</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH33" t="n">
+        <v>20</v>
+      </c>
+      <c r="AI33" t="n">
+        <v>35</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>21</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>74</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>430</v>
+      </c>
+      <c r="AO33" t="n">
+        <v>332</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>77.2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Everton</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>20</v>
+      </c>
+      <c r="F34" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" t="n">
+        <v>49</v>
+      </c>
+      <c r="H34" t="n">
+        <v>17</v>
+      </c>
+      <c r="I34" t="n">
+        <v>10</v>
+      </c>
+      <c r="J34" t="n">
+        <v>22</v>
+      </c>
+      <c r="K34" t="n">
+        <v>509</v>
+      </c>
+      <c r="L34" t="n">
+        <v>23</v>
+      </c>
+      <c r="M34" t="n">
+        <v>5</v>
+      </c>
+      <c r="N34" t="n">
+        <v>20</v>
+      </c>
+      <c r="O34" t="n">
+        <v>17</v>
+      </c>
+      <c r="P34" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>6</v>
+      </c>
+      <c r="R34" t="n">
+        <v>20</v>
+      </c>
+      <c r="S34" t="n">
+        <v>65</v>
+      </c>
+      <c r="T34" t="n">
+        <v>391</v>
+      </c>
+      <c r="U34" t="n">
+        <v>308</v>
+      </c>
+      <c r="V34" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="X34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>51</v>
+      </c>
+      <c r="AB34" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>523</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>16</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH34" t="n">
+        <v>17</v>
+      </c>
+      <c r="AI34" t="n">
+        <v>23</v>
+      </c>
+      <c r="AJ34" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK34" t="n">
+        <v>16</v>
+      </c>
+      <c r="AL34" t="n">
+        <v>14</v>
+      </c>
+      <c r="AM34" t="n">
+        <v>55</v>
+      </c>
+      <c r="AN34" t="n">
+        <v>411</v>
+      </c>
+      <c r="AO34" t="n">
+        <v>329</v>
+      </c>
+      <c r="AP34" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Fulham</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" t="n">
+        <v>3</v>
+      </c>
+      <c r="G35" t="n">
+        <v>54</v>
+      </c>
+      <c r="H35" t="n">
+        <v>20</v>
+      </c>
+      <c r="I35" t="n">
+        <v>3</v>
+      </c>
+      <c r="J35" t="n">
+        <v>22</v>
+      </c>
+      <c r="K35" t="n">
+        <v>618</v>
+      </c>
+      <c r="L35" t="n">
+        <v>24</v>
+      </c>
+      <c r="M35" t="n">
+        <v>6</v>
+      </c>
+      <c r="N35" t="n">
+        <v>14</v>
+      </c>
+      <c r="O35" t="n">
+        <v>23</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>7</v>
+      </c>
+      <c r="R35" t="n">
+        <v>25</v>
+      </c>
+      <c r="S35" t="n">
+        <v>55</v>
+      </c>
+      <c r="T35" t="n">
+        <v>504</v>
+      </c>
+      <c r="U35" t="n">
+        <v>408</v>
+      </c>
+      <c r="V35" t="n">
+        <v>81</v>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>Leeds United</t>
+        </is>
+      </c>
+      <c r="X35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>46</v>
+      </c>
+      <c r="AB35" t="n">
+        <v>15</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>13</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>546</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>18</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>7</v>
+      </c>
+      <c r="AH35" t="n">
+        <v>18</v>
+      </c>
+      <c r="AI35" t="n">
+        <v>30</v>
+      </c>
+      <c r="AJ35" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK35" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL35" t="n">
+        <v>15</v>
+      </c>
+      <c r="AM35" t="n">
+        <v>61</v>
+      </c>
+      <c r="AN35" t="n">
+        <v>426</v>
+      </c>
+      <c r="AO35" t="n">
+        <v>332</v>
+      </c>
+      <c r="AP35" t="n">
+        <v>77.90000000000001</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Newcastle United</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>16</v>
+      </c>
+      <c r="F36" t="n">
+        <v>4</v>
+      </c>
+      <c r="G36" t="n">
+        <v>57</v>
+      </c>
+      <c r="H36" t="n">
+        <v>10</v>
+      </c>
+      <c r="I36" t="n">
+        <v>9</v>
+      </c>
+      <c r="J36" t="n">
+        <v>25</v>
+      </c>
+      <c r="K36" t="n">
+        <v>618</v>
+      </c>
+      <c r="L36" t="n">
+        <v>10</v>
+      </c>
+      <c r="M36" t="n">
+        <v>6</v>
+      </c>
+      <c r="N36" t="n">
+        <v>21</v>
+      </c>
+      <c r="O36" t="n">
+        <v>20</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>8</v>
+      </c>
+      <c r="R36" t="n">
+        <v>28</v>
+      </c>
+      <c r="S36" t="n">
+        <v>69</v>
+      </c>
+      <c r="T36" t="n">
+        <v>509</v>
+      </c>
+      <c r="U36" t="n">
+        <v>400</v>
+      </c>
+      <c r="V36" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>Wolverhampton Wanderers</t>
+        </is>
+      </c>
+      <c r="X36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>43</v>
+      </c>
+      <c r="AB36" t="n">
+        <v>17</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>15</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>521</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>16</v>
+      </c>
+      <c r="AG36" t="n">
+        <v>14</v>
+      </c>
+      <c r="AH36" t="n">
+        <v>13</v>
+      </c>
+      <c r="AI36" t="n">
+        <v>38</v>
+      </c>
+      <c r="AJ36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK36" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL36" t="n">
+        <v>18</v>
+      </c>
+      <c r="AM36" t="n">
+        <v>81</v>
+      </c>
+      <c r="AN36" t="n">
+        <v>384</v>
+      </c>
+      <c r="AO36" t="n">
+        <v>286</v>
+      </c>
+      <c r="AP36" t="n">
+        <v>74.5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Bournemouth</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" t="n">
+        <v>12</v>
+      </c>
+      <c r="F37" t="n">
+        <v>4</v>
+      </c>
+      <c r="G37" t="n">
+        <v>51</v>
+      </c>
+      <c r="H37" t="n">
+        <v>16</v>
+      </c>
+      <c r="I37" t="n">
+        <v>4</v>
+      </c>
+      <c r="J37" t="n">
+        <v>19</v>
+      </c>
+      <c r="K37" t="n">
+        <v>560</v>
+      </c>
+      <c r="L37" t="n">
+        <v>18</v>
+      </c>
+      <c r="M37" t="n">
+        <v>3</v>
+      </c>
+      <c r="N37" t="n">
+        <v>17</v>
+      </c>
+      <c r="O37" t="n">
+        <v>37</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>12</v>
+      </c>
+      <c r="R37" t="n">
+        <v>17</v>
+      </c>
+      <c r="S37" t="n">
+        <v>70</v>
+      </c>
+      <c r="T37" t="n">
+        <v>434</v>
+      </c>
+      <c r="U37" t="n">
+        <v>330</v>
+      </c>
+      <c r="V37" t="n">
+        <v>76</v>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>Brighton &amp; Hove Albion</t>
+        </is>
+      </c>
+      <c r="X37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>49</v>
+      </c>
+      <c r="AB37" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>17</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>544</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>20</v>
+      </c>
+      <c r="AG37" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH37" t="n">
+        <v>9</v>
+      </c>
+      <c r="AI37" t="n">
+        <v>36</v>
+      </c>
+      <c r="AJ37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK37" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL37" t="n">
+        <v>20</v>
+      </c>
+      <c r="AM37" t="n">
+        <v>63</v>
+      </c>
+      <c r="AN37" t="n">
+        <v>415</v>
+      </c>
+      <c r="AO37" t="n">
+        <v>314</v>
+      </c>
+      <c r="AP37" t="n">
+        <v>75.7</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>West Ham United</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>7</v>
+      </c>
+      <c r="F38" t="n">
+        <v>4</v>
+      </c>
+      <c r="G38" t="n">
+        <v>36</v>
+      </c>
+      <c r="H38" t="n">
+        <v>8</v>
+      </c>
+      <c r="I38" t="n">
+        <v>2</v>
+      </c>
+      <c r="J38" t="n">
+        <v>9</v>
+      </c>
+      <c r="K38" t="n">
+        <v>454</v>
+      </c>
+      <c r="L38" t="n">
+        <v>13</v>
+      </c>
+      <c r="M38" t="n">
+        <v>5</v>
+      </c>
+      <c r="N38" t="n">
+        <v>22</v>
+      </c>
+      <c r="O38" t="n">
+        <v>40</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>9</v>
+      </c>
+      <c r="R38" t="n">
+        <v>19</v>
+      </c>
+      <c r="S38" t="n">
+        <v>66</v>
+      </c>
+      <c r="T38" t="n">
+        <v>340</v>
+      </c>
+      <c r="U38" t="n">
+        <v>262</v>
+      </c>
+      <c r="V38" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="X38" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>14</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>64</v>
+      </c>
+      <c r="AB38" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>13</v>
+      </c>
+      <c r="AD38" t="n">
+        <v>31</v>
+      </c>
+      <c r="AE38" t="n">
+        <v>678</v>
+      </c>
+      <c r="AF38" t="n">
+        <v>16</v>
+      </c>
+      <c r="AG38" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH38" t="n">
+        <v>13</v>
+      </c>
+      <c r="AI38" t="n">
+        <v>10</v>
+      </c>
+      <c r="AJ38" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK38" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL38" t="n">
+        <v>21</v>
+      </c>
+      <c r="AM38" t="n">
+        <v>62</v>
+      </c>
+      <c r="AN38" t="n">
+        <v>595</v>
+      </c>
+      <c r="AO38" t="n">
+        <v>493</v>
+      </c>
+      <c r="AP38" t="n">
+        <v>82.90000000000001</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-09-13</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Brentford</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" t="n">
+        <v>7</v>
+      </c>
+      <c r="F39" t="n">
+        <v>4</v>
+      </c>
+      <c r="G39" t="n">
+        <v>34</v>
+      </c>
+      <c r="H39" t="n">
+        <v>13</v>
+      </c>
+      <c r="I39" t="n">
+        <v>5</v>
+      </c>
+      <c r="J39" t="n">
+        <v>18</v>
+      </c>
+      <c r="K39" t="n">
+        <v>446</v>
+      </c>
+      <c r="L39" t="n">
+        <v>17</v>
+      </c>
+      <c r="M39" t="n">
+        <v>6</v>
+      </c>
+      <c r="N39" t="n">
+        <v>7</v>
+      </c>
+      <c r="O39" t="n">
+        <v>32</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>7</v>
+      </c>
+      <c r="R39" t="n">
+        <v>15</v>
+      </c>
+      <c r="S39" t="n">
+        <v>66</v>
+      </c>
+      <c r="T39" t="n">
+        <v>324</v>
+      </c>
+      <c r="U39" t="n">
+        <v>236</v>
+      </c>
+      <c r="V39" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="X39" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>66</v>
+      </c>
+      <c r="AB39" t="n">
+        <v>9</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>17</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>735</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>15</v>
+      </c>
+      <c r="AG39" t="n">
+        <v>13</v>
+      </c>
+      <c r="AH39" t="n">
+        <v>14</v>
+      </c>
+      <c r="AI39" t="n">
+        <v>34</v>
+      </c>
+      <c r="AJ39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AK39" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL39" t="n">
+        <v>20</v>
+      </c>
+      <c r="AM39" t="n">
+        <v>55</v>
+      </c>
+      <c r="AN39" t="n">
+        <v>617</v>
+      </c>
+      <c r="AO39" t="n">
+        <v>543</v>
+      </c>
+      <c r="AP39" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Burnley</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>20</v>
+      </c>
+      <c r="H40" t="n">
+        <v>9</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" t="n">
+        <v>3</v>
+      </c>
+      <c r="K40" t="n">
+        <v>320</v>
+      </c>
+      <c r="L40" t="n">
+        <v>16</v>
+      </c>
+      <c r="M40" t="n">
+        <v>17</v>
+      </c>
+      <c r="N40" t="n">
+        <v>16</v>
+      </c>
+      <c r="O40" t="n">
+        <v>46</v>
+      </c>
+      <c r="P40" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>21</v>
+      </c>
+      <c r="R40" t="n">
+        <v>11</v>
+      </c>
+      <c r="S40" t="n">
+        <v>68</v>
+      </c>
+      <c r="T40" t="n">
+        <v>189</v>
+      </c>
+      <c r="U40" t="n">
+        <v>87</v>
+      </c>
+      <c r="V40" t="n">
+        <v>46</v>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>Liverpool</t>
+        </is>
+      </c>
+      <c r="X40" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>26</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA40" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB40" t="n">
+        <v>9</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>13</v>
+      </c>
+      <c r="AD40" t="n">
+        <v>44</v>
+      </c>
+      <c r="AE40" t="n">
+        <v>868</v>
+      </c>
+      <c r="AF40" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG40" t="n">
+        <v>7</v>
+      </c>
+      <c r="AH40" t="n">
+        <v>27</v>
+      </c>
+      <c r="AI40" t="n">
+        <v>12</v>
+      </c>
+      <c r="AJ40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK40" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL40" t="n">
+        <v>21</v>
+      </c>
+      <c r="AM40" t="n">
+        <v>51</v>
+      </c>
+      <c r="AN40" t="n">
+        <v>766</v>
+      </c>
+      <c r="AO40" t="n">
+        <v>644</v>
+      </c>
+      <c r="AP40" t="n">
+        <v>84.09999999999999</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
+        <v>13</v>
+      </c>
+      <c r="F41" t="n">
+        <v>6</v>
+      </c>
+      <c r="G41" t="n">
+        <v>46</v>
+      </c>
+      <c r="H41" t="n">
+        <v>8</v>
+      </c>
+      <c r="I41" t="n">
+        <v>2</v>
+      </c>
+      <c r="J41" t="n">
+        <v>2</v>
+      </c>
+      <c r="K41" t="n">
+        <v>587</v>
+      </c>
+      <c r="L41" t="n">
+        <v>13</v>
+      </c>
+      <c r="M41" t="n">
+        <v>10</v>
+      </c>
+      <c r="N41" t="n">
+        <v>18</v>
+      </c>
+      <c r="O41" t="n">
+        <v>31</v>
+      </c>
+      <c r="P41" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>8</v>
+      </c>
+      <c r="R41" t="n">
+        <v>26</v>
+      </c>
+      <c r="S41" t="n">
+        <v>66</v>
+      </c>
+      <c r="T41" t="n">
+        <v>463</v>
+      </c>
+      <c r="U41" t="n">
+        <v>377</v>
+      </c>
+      <c r="V41" t="n">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="X41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>12</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA41" t="n">
+        <v>54</v>
+      </c>
+      <c r="AB41" t="n">
+        <v>8</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>4</v>
+      </c>
+      <c r="AD41" t="n">
+        <v>23</v>
+      </c>
+      <c r="AE41" t="n">
+        <v>653</v>
+      </c>
+      <c r="AF41" t="n">
+        <v>23</v>
+      </c>
+      <c r="AG41" t="n">
+        <v>13</v>
+      </c>
+      <c r="AH41" t="n">
+        <v>11</v>
+      </c>
+      <c r="AI41" t="n">
+        <v>10</v>
+      </c>
+      <c r="AJ41" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK41" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL41" t="n">
+        <v>21</v>
+      </c>
+      <c r="AM41" t="n">
+        <v>71</v>
+      </c>
+      <c r="AN41" t="n">
+        <v>550</v>
+      </c>
+      <c r="AO41" t="n">
+        <v>442</v>
+      </c>
+      <c r="AP41" t="n">
+        <v>80.40000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>